<commit_message>
Doi soat bao cao + bang theo so lieu VIVOS that, don dep repo
- Dong bo TASK2_REPORT.md/html va 2 bang (paper_vs_experiment, version_progress) theo ket qua that (V3 best: WER 43.30 / BLEU 22.73)

- Them configs/quick.yaml, code e2e (train_e2e, evaluate_e2e), manifests quick, notebook EDA

- Go cac file huong dan noi bo, tai lieu trung va thu muc submission khoi git

- Sua .gitignore: bao ve .env/logs/tensorboard, bo chan nham quick.yaml
</commit_message>
<xml_diff>
--- a/docs/version_progress.xlsx
+++ b/docs/version_progress.xlsx
@@ -440,16 +440,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.2" customWidth="1" min="1" max="1"/>
-    <col width="62.4" customWidth="1" min="2" max="2"/>
-    <col width="45.6" customWidth="1" min="3" max="3"/>
-    <col width="13.2" customWidth="1" min="4" max="4"/>
-    <col width="32.4" customWidth="1" min="5" max="5"/>
-    <col width="14.4" customWidth="1" min="6" max="6"/>
-    <col width="16.8" customWidth="1" min="7" max="7"/>
-    <col width="8.4" customWidth="1" min="8" max="8"/>
+    <col width="61.2" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
+    <col width="14.4" customWidth="1" min="4" max="4"/>
+    <col width="14.4" customWidth="1" min="5" max="5"/>
+    <col width="15.6" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="7.199999999999999" customWidth="1" min="8" max="8"/>
     <col width="33.6" customWidth="1" min="9" max="9"/>
-    <col width="42" customWidth="1" min="10" max="10"/>
-    <col width="32.4" customWidth="1" min="11" max="11"/>
+    <col width="46.8" customWidth="1" min="10" max="10"/>
+    <col width="43.2" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,22 +470,22 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>WER (dev)</t>
+          <t>WER (test)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>CER (dev)</t>
+          <t>CER (test)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>BLEU (dev)</t>
+          <t>BLEU (test)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>chrF++ (dev)</t>
+          <t>chrF++ (test)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -513,54 +513,50 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Whisper zero-shot + MarianMT cascade</t>
+          <t>Fine-tune Whisper-small, không augment, greedy</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Baseline để so sánh</t>
+          <t>Mốc tham chiếu trên audio thật</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>5130.77</t>
+          <t>50.52</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>5414.29</t>
+          <t>22.83</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>4.83</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>0.30</t>
+          <t>25.52</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>7.80</t>
+          <t>0.23</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>241M</t>
+          <t>241M + 77M</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Data quá kém</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> kết quả không có ý nghĩa</t>
-        </is>
-      </c>
+          <t>Mốc so sánh</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -570,40 +566,28 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Thêm augmentation (speed</t>
+          <t>+ Augmentation (speed/noise/reverb) + speaker cap</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> noise</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> reverb)</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Tăng robustness với nhiễu</t>
-        </is>
-      </c>
+          <t>Tăng robustness với biến thiên giọng/nhiễu - giảm WER</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>8.50</t>
-        </is>
-      </c>
+      <c r="I3" s="3" t="inlineStr"/>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>241M</t>
+          <t>241M + 77M</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Cải thiện nhỏ (dự đoán)</t>
+          <t>Đã huấn luyện - chưa chạy đánh giá</t>
         </is>
       </c>
     </row>
@@ -615,33 +599,49 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>LoRA fine-tune + beam search</t>
+          <t>+ LoRA (r=16) + beam search (size 5) + augment</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Tính hiệu + decode tốt hơn</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
-      <c r="F4" s="3" t="inlineStr"/>
+          <t>Fine-tune hiệu quả với ít VRAM; beam giảm lỗi decode</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>41.24</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>16.05</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>22.01</t>
+        </is>
+      </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>9.00</t>
+          <t>42.98</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>241M</t>
+          <t>0.27</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Cải thiện rõ hơn (dự đoán)</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="n"/>
+          <t>241M (~5M trainable) + 77M</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>WER tốt nhất; BLEU tăng ~4.6x</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="n"/>
     </row>
     <row r="5">
@@ -652,33 +652,49 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Noise-robust MT (fine-tune trên noisy transcripts)</t>
+          <t>+ Noise-robust MT + LoRA + beam</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Giảm lỗi lan truyền ASR→MT</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
+          <t>MT chịu lỗi ASR tốt hơn - giảm error propagation</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>43.30</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>16.88</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>22.73</t>
+        </is>
+      </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>9.50</t>
+          <t>43.62</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>241M</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>MT tốt hơn (dự đoán)</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="n"/>
+          <t>241M (~5M trainable) + 77M</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>BLEU/chrF++ tốt nhất - phiên bản chọn</t>
+        </is>
+      </c>
       <c r="K5" s="2" t="n"/>
     </row>
     <row r="6">
@@ -689,33 +705,41 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>End-to-end Whisper translation</t>
+          <t>End-to-end Whisper task=translate (bỏ MT)</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Đơn giản hóa pipeline</t>
+          <t>Kiểm chứng E2E vs cascade (đối chứng âm)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>4.23</t>
+        </is>
+      </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>8.00</t>
+          <t>17.21</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
+          <t>0.18</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
           <t>241M</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>Đơn giản hơn (dự đoán)</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="n"/>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Thất bại - kém cascade rõ rệt</t>
+        </is>
+      </c>
       <c r="K6" s="2" t="n"/>
     </row>
     <row r="7">
@@ -726,47 +750,47 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>V4 với data thật (VIVOS)</t>
+          <t>V3 (noise-robust MT + LoRA + beam)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Dùng data thật để có kết quả thực tế</t>
+          <t>Phiên bản tốt nhất để demo</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>~25.0</t>
+          <t>43.30</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>~15.0</t>
+          <t>16.88</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>~30.0</t>
+          <t>22.73</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>~0.6</t>
+          <t>43.62</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>~0.05</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>241M</t>
+          <t>241M + 77M</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Kết quả dự kiến tương đương paper</t>
+          <t>Chọn để demo</t>
         </is>
       </c>
       <c r="K7" s="2" t="n"/>

</xml_diff>